<commit_message>
chore: updated font formats
</commit_message>
<xml_diff>
--- a/AYAC 2026 Schedule of Events.xlsx
+++ b/AYAC 2026 Schedule of Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Israel Adefemi\Documents\Office\AYAC 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{566E798E-F6F3-4265-B776-7FC80B66742A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D84D42E-D368-42B9-9574-690549BF7F5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E09745D3-EC13-3B4E-8089-EA3CE444E0AC}"/>
   </bookViews>
@@ -540,28 +540,6 @@
   </si>
   <si>
     <r>
-      <t>Impartation, Holy Ghost Baptism &amp; Water Baptism</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">  </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(6:00am - 12:00pm)</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <rPr>
         <b/>
         <sz val="11"/>
@@ -694,7 +672,36 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">AYAC Prayer Hour </t>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Impartation, Holy Ghost Baptism &amp; Water Baptism</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(6:00am - 12:00pm)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">AYAC Prayer Hour  </t>
     </r>
     <r>
       <rPr>
@@ -711,13 +718,19 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -776,7 +789,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -819,6 +832,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="29">
     <border>
@@ -1180,218 +1199,218 @@
   </cellStyleXfs>
   <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1757,214 +1776,214 @@
   <sheetData>
     <row r="2" spans="3:14" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="3:14" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="8"/>
-      <c r="M3" s="8"/>
-      <c r="N3" s="9"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
+      <c r="K3" s="47"/>
+      <c r="L3" s="47"/>
+      <c r="M3" s="47"/>
+      <c r="N3" s="48"/>
     </row>
     <row r="4" spans="3:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="70" t="s">
+      <c r="C4" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="12"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="37"/>
+      <c r="H4" s="17"/>
       <c r="I4" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="J4" s="11" t="s">
+      <c r="J4" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="K4" s="12"/>
-      <c r="L4" s="11" t="s">
+      <c r="K4" s="17"/>
+      <c r="L4" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="M4" s="12"/>
+      <c r="M4" s="17"/>
       <c r="N4" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="3:14" ht="30" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C5" s="71" t="s">
+      <c r="C5" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="47"/>
-      <c r="F5" s="47"/>
-      <c r="G5" s="47"/>
-      <c r="H5" s="47"/>
-      <c r="I5" s="48"/>
-      <c r="J5" s="35" t="s">
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="65"/>
+      <c r="J5" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="36"/>
-      <c r="L5" s="37" t="s">
+      <c r="K5" s="35"/>
+      <c r="L5" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="M5" s="39" t="s">
+      <c r="M5" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="N5" s="38" t="s">
+      <c r="N5" s="53" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="6" spans="3:14" ht="91.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C6" s="69" t="s">
+      <c r="C6" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="72" t="s">
+      <c r="D6" s="60" t="s">
+        <v>54</v>
+      </c>
+      <c r="E6" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="E6" s="44" t="s">
+      <c r="F6" s="72" t="s">
+        <v>57</v>
+      </c>
+      <c r="G6" s="51" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="I6" s="71" t="s">
+        <v>49</v>
+      </c>
+      <c r="J6" s="66" t="s">
+        <v>39</v>
+      </c>
+      <c r="K6" s="56" t="s">
+        <v>30</v>
+      </c>
+      <c r="L6" s="38" t="s">
+        <v>41</v>
+      </c>
+      <c r="M6" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="N6" s="54"/>
+    </row>
+    <row r="7" spans="3:14" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="50"/>
+      <c r="D7" s="61"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="52"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="58"/>
+      <c r="J7" s="67"/>
+      <c r="K7" s="57"/>
+      <c r="L7" s="39"/>
+      <c r="M7" s="41"/>
+      <c r="N7" s="54"/>
+    </row>
+    <row r="8" spans="3:14" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C8" s="49" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="61"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="51" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" s="23"/>
+      <c r="I8" s="58"/>
+      <c r="J8" s="67"/>
+      <c r="K8" s="57"/>
+      <c r="L8" s="42" t="s">
+        <v>19</v>
+      </c>
+      <c r="M8" s="44" t="s">
+        <v>45</v>
+      </c>
+      <c r="N8" s="54"/>
+    </row>
+    <row r="9" spans="3:14" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C9" s="50"/>
+      <c r="D9" s="61"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="52"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="59"/>
+      <c r="J9" s="67"/>
+      <c r="K9" s="57"/>
+      <c r="L9" s="43"/>
+      <c r="M9" s="45"/>
+      <c r="N9" s="54"/>
+    </row>
+    <row r="10" spans="3:14" ht="136.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C10" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="61"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="51" t="s">
+        <v>46</v>
+      </c>
+      <c r="H10" s="23"/>
+      <c r="I10" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="J10" s="67"/>
+      <c r="K10" s="57"/>
+      <c r="L10" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="M10" s="29"/>
+      <c r="N10" s="54"/>
+    </row>
+    <row r="11" spans="3:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C11" s="20"/>
+      <c r="D11" s="62"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="33"/>
+      <c r="G11" s="52"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="41"/>
+      <c r="J11" s="67"/>
+      <c r="K11" s="57"/>
+      <c r="L11" s="30"/>
+      <c r="M11" s="31"/>
+      <c r="N11" s="55"/>
+    </row>
+    <row r="12" spans="3:14" ht="128.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C12" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="70" t="s">
         <v>56</v>
       </c>
-      <c r="F6" s="56" t="s">
-        <v>57</v>
-      </c>
-      <c r="G6" s="49" t="s">
-        <v>43</v>
-      </c>
-      <c r="H6" s="43" t="s">
-        <v>49</v>
-      </c>
-      <c r="I6" s="49" t="s">
-        <v>50</v>
-      </c>
-      <c r="J6" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="K6" s="54" t="s">
-        <v>30</v>
-      </c>
-      <c r="L6" s="20" t="s">
-        <v>41</v>
-      </c>
-      <c r="M6" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="N6" s="22"/>
-    </row>
-    <row r="7" spans="3:14" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="10"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="57"/>
-      <c r="G7" s="50"/>
-      <c r="H7" s="44"/>
-      <c r="I7" s="51"/>
-      <c r="J7" s="55"/>
-      <c r="K7" s="34"/>
-      <c r="L7" s="21"/>
-      <c r="M7" s="24"/>
-      <c r="N7" s="22"/>
-    </row>
-    <row r="8" spans="3:14" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C8" s="69" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="40"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="57"/>
-      <c r="G8" s="49" t="s">
-        <v>44</v>
-      </c>
-      <c r="H8" s="44"/>
-      <c r="I8" s="51"/>
-      <c r="J8" s="55"/>
-      <c r="K8" s="34"/>
-      <c r="L8" s="25" t="s">
-        <v>19</v>
-      </c>
-      <c r="M8" s="27" t="s">
-        <v>45</v>
-      </c>
-      <c r="N8" s="22"/>
-    </row>
-    <row r="9" spans="3:14" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="10"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="44"/>
-      <c r="F9" s="57"/>
-      <c r="G9" s="50"/>
-      <c r="H9" s="44"/>
-      <c r="I9" s="52"/>
-      <c r="J9" s="55"/>
-      <c r="K9" s="34"/>
-      <c r="L9" s="26"/>
-      <c r="M9" s="28"/>
-      <c r="N9" s="22"/>
-    </row>
-    <row r="10" spans="3:14" ht="136.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C10" s="67" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="40"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="57"/>
-      <c r="G10" s="49" t="s">
-        <v>46</v>
-      </c>
-      <c r="H10" s="44"/>
-      <c r="I10" s="23" t="s">
+      <c r="E12" s="69"/>
+      <c r="F12" s="69"/>
+      <c r="G12" s="69"/>
+      <c r="H12" s="69"/>
+      <c r="I12" s="69"/>
+      <c r="J12" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="J10" s="55"/>
-      <c r="K10" s="34"/>
-      <c r="L10" s="60" t="s">
-        <v>48</v>
-      </c>
-      <c r="M10" s="29"/>
-      <c r="N10" s="22"/>
-    </row>
-    <row r="11" spans="3:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C11" s="68"/>
-      <c r="D11" s="41"/>
-      <c r="E11" s="45"/>
-      <c r="F11" s="58"/>
-      <c r="G11" s="50"/>
-      <c r="H11" s="45"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="55"/>
-      <c r="K11" s="34"/>
-      <c r="L11" s="61"/>
-      <c r="M11" s="62"/>
-      <c r="N11" s="63"/>
-    </row>
-    <row r="12" spans="3:14" ht="128.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="71" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" s="59" t="s">
-        <v>47</v>
-      </c>
-      <c r="E12" s="42"/>
-      <c r="F12" s="42"/>
-      <c r="G12" s="42"/>
-      <c r="H12" s="42"/>
-      <c r="I12" s="42"/>
-      <c r="J12" s="64" t="s">
-        <v>52</v>
-      </c>
-      <c r="K12" s="65"/>
-      <c r="L12" s="65"/>
-      <c r="M12" s="65"/>
-      <c r="N12" s="66"/>
+      <c r="K12" s="26"/>
+      <c r="L12" s="26"/>
+      <c r="M12" s="26"/>
+      <c r="N12" s="27"/>
     </row>
     <row r="16" spans="3:14" ht="30" x14ac:dyDescent="0.25">
       <c r="C16" s="5" t="s">
@@ -1974,11 +1993,11 @@
         <v>2</v>
       </c>
       <c r="E16" s="2"/>
-      <c r="F16" s="14" t="s">
+      <c r="F16" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="G16" s="14"/>
-      <c r="H16" s="17"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="7"/>
     </row>
     <row r="17" spans="3:9" ht="15" x14ac:dyDescent="0.25">
       <c r="C17" s="3" t="s">
@@ -1987,11 +2006,11 @@
       <c r="D17" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F17" s="15" t="s">
+      <c r="F17" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="G17" s="15"/>
-      <c r="H17" s="18"/>
+      <c r="G17" s="21"/>
+      <c r="H17" s="8"/>
       <c r="I17" s="4"/>
     </row>
     <row r="18" spans="3:9" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2001,158 +2020,139 @@
       <c r="D18" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F18" s="16" t="s">
+      <c r="F18" s="68" t="s">
         <v>10</v>
       </c>
-      <c r="G18" s="16"/>
-      <c r="H18" s="19"/>
+      <c r="G18" s="68"/>
+      <c r="H18" s="9"/>
       <c r="I18" s="4"/>
     </row>
     <row r="19" spans="3:9" ht="29.25" x14ac:dyDescent="0.25">
-      <c r="C19" s="31" t="s">
+      <c r="C19" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D19" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="D19" s="31" t="s">
-        <v>54</v>
-      </c>
-      <c r="F19" s="15" t="s">
+      <c r="F19" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="G19" s="15"/>
-      <c r="H19" s="18"/>
+      <c r="G19" s="21"/>
+      <c r="H19" s="8"/>
       <c r="I19" s="4"/>
     </row>
     <row r="20" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="F20" s="33" t="s">
+      <c r="F20" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G20" s="33"/>
-      <c r="H20" s="19"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="9"/>
       <c r="I20" s="4"/>
     </row>
     <row r="21" spans="3:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F21" s="33" t="s">
+      <c r="F21" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="G21" s="33"/>
-      <c r="H21" s="19"/>
+      <c r="G21" s="18"/>
+      <c r="H21" s="9"/>
       <c r="I21" s="4"/>
     </row>
     <row r="22" spans="3:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F22" s="33" t="s">
+      <c r="F22" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="G22" s="33"/>
-      <c r="H22" s="19"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="9"/>
       <c r="I22" s="4"/>
     </row>
     <row r="23" spans="3:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F23" s="33" t="s">
+      <c r="F23" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="G23" s="33"/>
-      <c r="H23" s="19"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="9"/>
       <c r="I23" s="4"/>
     </row>
     <row r="24" spans="3:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F24" s="33" t="s">
+      <c r="F24" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="G24" s="33"/>
-      <c r="H24" s="19"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="9"/>
       <c r="I24" s="4"/>
     </row>
     <row r="25" spans="3:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F25" s="33" t="s">
+      <c r="F25" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="G25" s="33"/>
-      <c r="H25" s="19"/>
+      <c r="G25" s="18"/>
+      <c r="H25" s="9"/>
       <c r="I25" s="4"/>
     </row>
     <row r="26" spans="3:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="F26" s="15" t="s">
+      <c r="F26" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="G26" s="15"/>
-      <c r="H26" s="19"/>
+      <c r="G26" s="21"/>
+      <c r="H26" s="9"/>
       <c r="I26" s="4"/>
     </row>
     <row r="27" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="F27" s="16" t="s">
+      <c r="F27" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="G27" s="16"/>
-      <c r="H27" s="19"/>
+      <c r="G27" s="68"/>
+      <c r="H27" s="9"/>
       <c r="I27" s="4"/>
     </row>
     <row r="28" spans="3:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="F28" s="16" t="s">
+      <c r="F28" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="G28" s="16"/>
-      <c r="H28" s="18"/>
+      <c r="G28" s="68"/>
+      <c r="H28" s="8"/>
       <c r="I28" s="4"/>
     </row>
     <row r="29" spans="3:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="F29" s="15" t="s">
+      <c r="F29" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="G29" s="15"/>
-      <c r="H29" s="19"/>
+      <c r="G29" s="21"/>
+      <c r="H29" s="9"/>
       <c r="I29" s="4"/>
     </row>
     <row r="30" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="F30" s="16" t="s">
+      <c r="F30" s="68" t="s">
         <v>12</v>
       </c>
-      <c r="G30" s="16"/>
-      <c r="H30" s="19"/>
+      <c r="G30" s="68"/>
+      <c r="H30" s="9"/>
       <c r="I30" s="4"/>
     </row>
     <row r="31" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="H31" s="19"/>
+      <c r="H31" s="9"/>
       <c r="I31" s="4"/>
     </row>
     <row r="32" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H32" s="30"/>
+      <c r="H32" s="2"/>
       <c r="I32" s="4"/>
     </row>
     <row r="33" spans="8:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H33" s="32"/>
+      <c r="H33" s="11"/>
     </row>
     <row r="34" spans="8:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H34" s="32"/>
+      <c r="H34" s="11"/>
     </row>
     <row r="35" spans="8:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H35" s="32"/>
+      <c r="H35" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="43">
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="E6:E11"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="D12:I12"/>
-    <mergeCell ref="J12:N12"/>
-    <mergeCell ref="L10:M11"/>
-    <mergeCell ref="F6:F11"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="H6:H11"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="L6:L7"/>
-    <mergeCell ref="M6:M7"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="F30:G30"/>
     <mergeCell ref="C3:N3"/>
     <mergeCell ref="C6:C7"/>
     <mergeCell ref="C8:C9"/>
@@ -2166,14 +2166,33 @@
     <mergeCell ref="D6:D11"/>
     <mergeCell ref="D5:I5"/>
     <mergeCell ref="J6:J11"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="D12:I12"/>
+    <mergeCell ref="J12:N12"/>
+    <mergeCell ref="L10:M11"/>
+    <mergeCell ref="F6:F11"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="H6:H11"/>
+    <mergeCell ref="D4:H4"/>
+    <mergeCell ref="L6:L7"/>
+    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="E6:E11"/>
     <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="F24:G24"/>
   </mergeCells>
-  <phoneticPr fontId="5" type="noConversion"/>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="48" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>

</xml_diff>